<commit_message>
implemented export to xls
</commit_message>
<xml_diff>
--- a/main/xls/stock_template.xlsx
+++ b/main/xls/stock_template.xlsx
@@ -8,15 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\python\vetis_tools\main\xls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777D72B6-62D7-463F-9E1D-4E19507AB773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E28089-EDE0-4483-839B-F05073556893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E00D4390-7223-4615-B085-48A3A81733E7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E00D4390-7223-4615-B085-48A3A81733E7}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
     <sheet name="Сводная" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">Сводная!$7:$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="261" r:id="rId3"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,8 +42,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
   <si>
     <t>ХС</t>
   </si>
@@ -118,6 +146,18 @@
   </si>
   <si>
     <t>Обновлено:</t>
+  </si>
+  <si>
+    <t>(Все)</t>
+  </si>
+  <si>
+    <t>Общий итог</t>
+  </si>
+  <si>
+    <t>Нерка Итог</t>
+  </si>
+  <si>
+    <t>_остаток</t>
   </si>
 </sst>
 </file>
@@ -127,7 +167,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,16 +176,70 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -153,20 +247,194 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" pivotButton="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" pivotButton="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="28">
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -216,25 +484,313 @@
 </styleSheet>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Pavel" refreshedDate="45985.596929861109" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{5539164E-E57E-4F01-9C4A-AADEE2F83270}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="stock_entries"/>
+  </cacheSource>
+  <cacheFields count="15">
+    <cacheField name="ХС" numFmtId="49">
+      <sharedItems count="1">
+        <s v="Меркурий"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Предприятие" numFmtId="49">
+      <sharedItems count="1">
+        <s v="ООО &quot;Меркурий&quot; (Российская Федерация, г. Севастополь, Хрусталева ул., д. здание 76ж/1, стр. 1)"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Номер записи" numFmtId="49">
+      <sharedItems count="1">
+        <s v="49093132205"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Дата поступления" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-05-22T00:00:00" maxDate="2024-05-23T00:00:00"/>
+    </cacheField>
+    <cacheField name="Статус" numFmtId="49">
+      <sharedItems count="1">
+        <s v="Гашение ВСД"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Наименование продукции" numFmtId="49">
+      <sharedItems count="1">
+        <s v="Мороженая пищевая рыбная продукция.Нерка дальневосточная потрошенная обезглавленная мороженая глазированная 1/20 кг"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="ЕИ" numFmtId="49">
+      <sharedItems count="1">
+        <s v="кг"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Объем" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="77" maxValue="77" count="1">
+        <n v="77"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Остаток" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="70.5" maxValue="70.5"/>
+    </cacheField>
+    <cacheField name="Выработано" numFmtId="49">
+      <sharedItems count="1">
+        <s v="12.07.2022 - 07.08.2022"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Годен до" numFmtId="49">
+      <sharedItems count="1">
+        <s v="07.08.2024"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Срок годности" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-08-07T00:00:00" maxDate="2024-08-08T00:00:00" count="1">
+        <d v="2024-08-07T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Источник" numFmtId="49">
+      <sharedItems count="1">
+        <s v="ЧЕРНОМОРЕЦ ИВАН ИВАНОВИЧ (561015332235) / ИП Черноморец Иван Иванович (Российская Федерация, г. Севастополь, Индустриальная ул., д. 16)"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Группа" numFmtId="49">
+      <sharedItems count="1">
+        <s v="Нерка"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Тип продукции" numFmtId="49">
+      <sharedItems count="1">
+        <s v="Рыба и морепродукты"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="1">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <d v="2024-05-22T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="70.5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0163A2FC-837D-49EA-A736-E14D9CF8FE9D}" name="Сводная таблица5" cacheId="261" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Значения" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A7:J10" firstHeaderRow="1" firstDataRow="1" firstDataCol="9" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="15">
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" sortType="ascending" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" numFmtId="14" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" numFmtId="14" outline="0" showAll="0" sortType="ascending" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="9">
+    <field x="13"/>
+    <field x="11"/>
+    <field x="2"/>
+    <field x="5"/>
+    <field x="12"/>
+    <field x="9"/>
+    <field x="10"/>
+    <field x="6"/>
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+      <x/>
+      <x/>
+      <x/>
+      <x/>
+      <x/>
+      <x/>
+      <x/>
+      <x/>
+    </i>
+    <i t="default">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="4" hier="-1"/>
+    <pageField fld="14" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="_остаток" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="15">
+    <format dxfId="15">
+      <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="13" count="0" defaultSubtotal="1"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea field="13" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="12">
+      <pivotArea field="11" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
+    </format>
+    <format dxfId="11">
+      <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="2"/>
+    </format>
+    <format dxfId="10">
+      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="3"/>
+    </format>
+    <format dxfId="9">
+      <pivotArea field="12" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="4"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea field="9" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="5"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="6"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="7"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="8"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="7" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CCE5EDC-E616-4323-8252-5B9BFC562F48}" name="stock_entries" displayName="stock_entries" ref="A3:O4" totalsRowShown="0">
   <autoFilter ref="A3:O4" xr:uid="{9CCE5EDC-E616-4323-8252-5B9BFC562F48}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{13394211-5500-42E1-A77B-D293BBEF5E7D}" name="ХС" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{D555ACB0-C6DB-4DAD-9FCB-0055E2D7F67E}" name="Предприятие" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{F58CC30E-00B0-404B-860A-041B951A39A2}" name="Номер записи" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{13394211-5500-42E1-A77B-D293BBEF5E7D}" name="ХС" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{D555ACB0-C6DB-4DAD-9FCB-0055E2D7F67E}" name="Предприятие" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{F58CC30E-00B0-404B-860A-041B951A39A2}" name="Номер записи" dataDxfId="25"/>
     <tableColumn id="4" xr3:uid="{1EB776CC-459B-413E-97C4-4E7B391D4ABD}" name="Дата поступления"/>
-    <tableColumn id="5" xr3:uid="{F5018B71-950D-42E0-B090-1AFFEE92A2B5}" name="Статус" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{BACC915B-588E-43D6-867A-E932EBF51052}" name="Наименование продукции" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{3BC7CCE2-1202-4EE2-AA33-5FF1AE612230}" name="ЕИ" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{F5018B71-950D-42E0-B090-1AFFEE92A2B5}" name="Статус" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{BACC915B-588E-43D6-867A-E932EBF51052}" name="Наименование продукции" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{3BC7CCE2-1202-4EE2-AA33-5FF1AE612230}" name="ЕИ" dataDxfId="22"/>
     <tableColumn id="8" xr3:uid="{E002A09B-902D-4864-A74B-8F4AF4FF9C7D}" name="Объем"/>
     <tableColumn id="9" xr3:uid="{3ACA75B5-E5E4-4281-9617-1B5DFD3028BC}" name="Остаток"/>
-    <tableColumn id="10" xr3:uid="{093C570C-71A0-4DF4-95AE-924C7C16EBB5}" name="Выработано" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{4AB3B47E-F1D0-48F3-945E-01AE0701D474}" name="Годен до" dataDxfId="4"/>
-    <tableColumn id="14" xr3:uid="{2B135885-3ECC-49AE-B3E1-42FEDD6EA3BC}" name="Срок годности" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{8902DB5E-9DCD-4CC5-8267-26F0CB697628}" name="Источник" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{FC77A379-66DB-4CD5-A3A7-F39BD9D81087}" name="Группа" dataDxfId="1"/>
-    <tableColumn id="15" xr3:uid="{12C7F003-DF72-4AAF-B3D8-5305C51288F6}" name="Тип продукции" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{093C570C-71A0-4DF4-95AE-924C7C16EBB5}" name="Выработано" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{4AB3B47E-F1D0-48F3-945E-01AE0701D474}" name="Годен до" dataDxfId="20"/>
+    <tableColumn id="14" xr3:uid="{2B135885-3ECC-49AE-B3E1-42FEDD6EA3BC}" name="Срок годности" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{8902DB5E-9DCD-4CC5-8267-26F0CB697628}" name="Источник" dataDxfId="18"/>
+    <tableColumn id="13" xr3:uid="{FC77A379-66DB-4CD5-A3A7-F39BD9D81087}" name="Группа" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{12C7F003-DF72-4AAF-B3D8-5305C51288F6}" name="Тип продукции" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -689,10 +1245,146 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5236A611-EE76-4704-8E1B-D0D9EBBCB502}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="49.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" customWidth="1"/>
+    <col min="6" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="str">
+        <f>"Складской журнал по состоянию на " &amp; TEXT(data!B1,"ДД.ММ.ГГГГ  ЧЧ:ММ")</f>
+        <v>Складской журнал по состоянию на 24.11.2025 12:00</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="str" cm="1">
+        <f t="array" ref="A2">stock_entries[Предприятие]</f>
+        <v>ООО "Меркурий" (Российская Федерация, г. Севастополь, Хрусталева ул., д. здание 76ж/1, стр. 1)</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="5">
+        <v>45511</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="15">
+        <v>77</v>
+      </c>
+      <c r="J8" s="16">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="17">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="18">
+        <v>70.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="68" fitToHeight="0" orientation="landscape" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add producer_name to xls export
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/main/xls/stock_template.xlsx
+++ b/main/xls/stock_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\python\vetis_tools\main\xls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E28089-EDE0-4483-839B-F05073556893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C32F1A8A-0476-4FAE-A304-BE20AC067B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E00D4390-7223-4615-B085-48A3A81733E7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E00D4390-7223-4615-B085-48A3A81733E7}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="261" r:id="rId3"/>
+    <pivotCache cacheId="237" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="32">
   <si>
     <t>ХС</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>_остаток</t>
+  </si>
+  <si>
+    <t>Производитель</t>
   </si>
 </sst>
 </file>
@@ -195,14 +198,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1" tint="0.499984740745262"/>
       <name val="Aptos Narrow"/>
@@ -216,6 +211,16 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -342,12 +347,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" pivotButton="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" pivotButton="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -356,7 +361,43 @@
   </cellStyles>
   <dxfs count="28">
     <dxf>
-      <alignment horizontal="right"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -434,42 +475,6 @@
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -485,7 +490,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Pavel" refreshedDate="45985.596929861109" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{5539164E-E57E-4F01-9C4A-AADEE2F83270}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Pavel" refreshedDate="45985.596929861109" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{5539164E-E57E-4F01-9C4A-AADEE2F83270}">
   <cacheSource type="worksheet">
     <worksheetSource name="stock_entries"/>
   </cacheSource>
@@ -593,7 +598,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0163A2FC-837D-49EA-A736-E14D9CF8FE9D}" name="Сводная таблица5" cacheId="261" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Значения" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0163A2FC-837D-49EA-A736-E14D9CF8FE9D}" name="Сводная таблица5" cacheId="237" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Значения" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A7:J10" firstHeaderRow="1" firstDataRow="1" firstDataCol="9" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="15">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -612,7 +617,7 @@
       </items>
     </pivotField>
     <pivotField compact="0" numFmtId="14" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" sortType="ascending" defaultSubtotal="0">
       <items count="1">
         <item x="0"/>
       </items>
@@ -659,7 +664,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" sortType="ascending" defaultSubtotal="0">
       <items count="1">
         <item x="0"/>
       </items>
@@ -706,57 +711,57 @@
     <dataField name="_остаток" fld="8" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="15">
-    <format dxfId="15">
+    <format dxfId="27">
       <pivotArea dataOnly="0" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="13" count="0" defaultSubtotal="1"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="26">
       <pivotArea dataOnly="0" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="25">
       <pivotArea field="13" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="24">
       <pivotArea field="11" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="23">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="2"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="22">
       <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="3"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="21">
       <pivotArea field="12" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="4"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="20">
       <pivotArea field="9" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="5"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="19">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="6"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="18">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="7"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="17">
       <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="8"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="7" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="14">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -773,24 +778,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CCE5EDC-E616-4323-8252-5B9BFC562F48}" name="stock_entries" displayName="stock_entries" ref="A3:O4" totalsRowShown="0">
-  <autoFilter ref="A3:O4" xr:uid="{9CCE5EDC-E616-4323-8252-5B9BFC562F48}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{13394211-5500-42E1-A77B-D293BBEF5E7D}" name="ХС" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{D555ACB0-C6DB-4DAD-9FCB-0055E2D7F67E}" name="Предприятие" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{F58CC30E-00B0-404B-860A-041B951A39A2}" name="Номер записи" dataDxfId="25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CCE5EDC-E616-4323-8252-5B9BFC562F48}" name="stock_entries" displayName="stock_entries" ref="A3:P4" totalsRowShown="0">
+  <autoFilter ref="A3:P4" xr:uid="{9CCE5EDC-E616-4323-8252-5B9BFC562F48}"/>
+  <tableColumns count="16">
+    <tableColumn id="1" xr3:uid="{13394211-5500-42E1-A77B-D293BBEF5E7D}" name="ХС" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{D555ACB0-C6DB-4DAD-9FCB-0055E2D7F67E}" name="Предприятие" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{F58CC30E-00B0-404B-860A-041B951A39A2}" name="Номер записи" dataDxfId="10"/>
     <tableColumn id="4" xr3:uid="{1EB776CC-459B-413E-97C4-4E7B391D4ABD}" name="Дата поступления"/>
-    <tableColumn id="5" xr3:uid="{F5018B71-950D-42E0-B090-1AFFEE92A2B5}" name="Статус" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{BACC915B-588E-43D6-867A-E932EBF51052}" name="Наименование продукции" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{3BC7CCE2-1202-4EE2-AA33-5FF1AE612230}" name="ЕИ" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{F5018B71-950D-42E0-B090-1AFFEE92A2B5}" name="Статус" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{BACC915B-588E-43D6-867A-E932EBF51052}" name="Наименование продукции" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{3BC7CCE2-1202-4EE2-AA33-5FF1AE612230}" name="ЕИ" dataDxfId="7"/>
     <tableColumn id="8" xr3:uid="{E002A09B-902D-4864-A74B-8F4AF4FF9C7D}" name="Объем"/>
     <tableColumn id="9" xr3:uid="{3ACA75B5-E5E4-4281-9617-1B5DFD3028BC}" name="Остаток"/>
-    <tableColumn id="10" xr3:uid="{093C570C-71A0-4DF4-95AE-924C7C16EBB5}" name="Выработано" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{4AB3B47E-F1D0-48F3-945E-01AE0701D474}" name="Годен до" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{2B135885-3ECC-49AE-B3E1-42FEDD6EA3BC}" name="Срок годности" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{8902DB5E-9DCD-4CC5-8267-26F0CB697628}" name="Источник" dataDxfId="18"/>
-    <tableColumn id="13" xr3:uid="{FC77A379-66DB-4CD5-A3A7-F39BD9D81087}" name="Группа" dataDxfId="17"/>
-    <tableColumn id="15" xr3:uid="{12C7F003-DF72-4AAF-B3D8-5305C51288F6}" name="Тип продукции" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{093C570C-71A0-4DF4-95AE-924C7C16EBB5}" name="Выработано" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{4AB3B47E-F1D0-48F3-945E-01AE0701D474}" name="Годен до" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{2B135885-3ECC-49AE-B3E1-42FEDD6EA3BC}" name="Срок годности" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{8902DB5E-9DCD-4CC5-8267-26F0CB697628}" name="Источник" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{81ECCFA2-A7BE-414F-A5BA-6E93C99B7DE5}" name="Производитель" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{FC77A379-66DB-4CD5-A3A7-F39BD9D81087}" name="Группа" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{12C7F003-DF72-4AAF-B3D8-5305C51288F6}" name="Тип продукции" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1113,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3586547-A36A-4FE4-8D01-ED1B417BAACB}">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" customWidth="1"/>
@@ -1126,12 +1132,12 @@
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="10.42578125" customWidth="1"/>
     <col min="10" max="12" width="15.140625" customWidth="1"/>
-    <col min="13" max="13" width="32" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" customWidth="1"/>
+    <col min="13" max="13" width="28.7109375" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
     <col min="15" max="15" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -1139,7 +1145,7 @@
         <v>45985.500173611108</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1180,13 +1186,16 @@
         <v>5</v>
       </c>
       <c r="N3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" t="s">
         <v>2</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1227,9 +1236,12 @@
         <v>21</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1288,31 +1300,31 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="15" t="s">
         <v>12</v>
       </c>
       <c r="J7" s="19" t="s">
@@ -1344,7 +1356,7 @@
       <c r="H8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="14">
         <v>77</v>
       </c>
       <c r="J8" s="16">

</xml_diff>